<commit_message>
Update .csv and .xlsx files with the Danish cities
</commit_message>
<xml_diff>
--- a/cities/development/european_100000pop_comments.xlsx
+++ b/cities/development/european_100000pop_comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianapessoa/Desktop/dataexport/cities/development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF10DB0-4617-E849-A683-EE4D60F8E236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D2CFBB-A902-374B-AF4F-62C186A0699D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2469,7 +2469,7 @@
         <v>557</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
@@ -2495,7 +2495,7 @@
         <v>557</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
@@ -5413,7 +5413,7 @@
         <v>557</v>
       </c>
       <c r="H123">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.2">
@@ -12970,7 +12970,7 @@
         <v>557</v>
       </c>
       <c r="H428">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>